<commit_message>
solution to the problem
</commit_message>
<xml_diff>
--- a/100040000/raw_data.xlsx
+++ b/100040000/raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carcheme\PycharmProjects\gyan\mini_project\100040000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carla\clariant\mini_project\100040000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F067EA4-E8EE-46AE-A04B-D9CB8E2E19D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4566407-094A-494F-8B79-2EF56B9672DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1830" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{83AC14B2-2E1F-4BB3-8D35-B9BFFD3D8107}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{83AC14B2-2E1F-4BB3-8D35-B9BFFD3D8107}"/>
   </bookViews>
   <sheets>
     <sheet name="2-122941" sheetId="6" r:id="rId1"/>
@@ -85,12 +85,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -125,12 +131,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1452,7 +1459,7 @@
         <c:crossAx val="838029408"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
-        <c:majorUnit val="2"/>
+        <c:majorUnit val="1"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="838029408"/>
@@ -4664,6 +4671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E184353-1CFB-446A-A81A-D18C23793B52}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -6430,6 +6438,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500452F6-1F54-4F14-A3A1-965B9FE55121}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:L200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -8220,6 +8229,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A7B6B71-1464-4720-A6A3-1B702730BA59}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:K200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -8335,7 +8345,7 @@
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>3.1859999999999999</v>
       </c>
       <c r="H5">
@@ -8355,7 +8365,7 @@
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>3.3239999999999998</v>
       </c>
       <c r="H6">
@@ -8594,7 +8604,7 @@
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>2.2469999999999999</v>
       </c>
     </row>
@@ -8826,7 +8836,7 @@
       <c r="A52">
         <v>52</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="3">
         <v>3.5089999999999999</v>
       </c>
     </row>
@@ -8914,7 +8924,7 @@
       <c r="A63">
         <v>63</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="3">
         <v>2.2389999999999999</v>
       </c>
     </row>
@@ -8922,7 +8932,7 @@
       <c r="A64">
         <v>64</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="3">
         <v>2.819</v>
       </c>
     </row>
@@ -8946,7 +8956,7 @@
       <c r="A67">
         <v>67</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="3">
         <v>2.7970000000000002</v>
       </c>
     </row>
@@ -8954,7 +8964,7 @@
       <c r="A68">
         <v>68</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="3">
         <v>3.7170000000000001</v>
       </c>
     </row>
@@ -9106,7 +9116,7 @@
       <c r="A87">
         <v>87</v>
       </c>
-      <c r="B87">
+      <c r="B87" s="3">
         <v>2.819</v>
       </c>
     </row>
@@ -9202,7 +9212,7 @@
       <c r="A99">
         <v>99</v>
       </c>
-      <c r="B99">
+      <c r="B99" s="3">
         <v>3.8279999999999998</v>
       </c>
     </row>
@@ -9346,7 +9356,7 @@
       <c r="A117">
         <v>117</v>
       </c>
-      <c r="B117">
+      <c r="B117" s="3">
         <v>3.9460000000000002</v>
       </c>
     </row>
@@ -9410,7 +9420,7 @@
       <c r="A125">
         <v>125</v>
       </c>
-      <c r="B125">
+      <c r="B125" s="3">
         <v>3.8279999999999998</v>
       </c>
     </row>
@@ -9822,7 +9832,7 @@
         <v>10.49</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>177</v>
       </c>
@@ -9830,7 +9840,7 @@
         <v>11.831</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>178</v>
       </c>
@@ -9838,7 +9848,7 @@
         <v>8.3989999999999991</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>179</v>
       </c>
@@ -9846,7 +9856,7 @@
         <v>8.1630000000000003</v>
       </c>
     </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>180</v>
       </c>
@@ -9854,7 +9864,7 @@
         <v>9.7899999999999991</v>
       </c>
     </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>181</v>
       </c>
@@ -9862,7 +9872,7 @@
         <v>7.0019999999999998</v>
       </c>
     </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>182</v>
       </c>
@@ -9870,7 +9880,7 @@
         <v>6.7169999999999996</v>
       </c>
     </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>183</v>
       </c>
@@ -9878,7 +9888,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>184</v>
       </c>
@@ -9886,7 +9896,7 @@
         <v>4.8570000000000002</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>185</v>
       </c>
@@ -9894,7 +9904,7 @@
         <v>8.0500000000000007</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>186</v>
       </c>
@@ -9902,7 +9912,7 @@
         <v>8.7479999999999993</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>187</v>
       </c>
@@ -9910,15 +9920,18 @@
         <v>8.6359999999999992</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>188</v>
       </c>
       <c r="B188">
         <v>5.4619999999999997</v>
       </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E188">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>189</v>
       </c>
@@ -9926,7 +9939,7 @@
         <v>8.2520000000000007</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>190</v>
       </c>
@@ -9934,7 +9947,7 @@
         <v>7.2080000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>191</v>
       </c>
@@ -9942,7 +9955,7 @@
         <v>11.106999999999999</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>192</v>
       </c>

</xml_diff>